<commit_message>
added close day book option
</commit_message>
<xml_diff>
--- a/files/reconsilationfornmat.xlsx
+++ b/files/reconsilationfornmat.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="87">
   <si>
     <t>BLOCK</t>
   </si>
@@ -59,46 +59,46 @@
     <t>no</t>
   </si>
   <si>
+    <t>DIGSIRA</t>
+  </si>
+  <si>
+    <t>GHANTABAHALI</t>
+  </si>
+  <si>
+    <t>GHODAR</t>
+  </si>
+  <si>
+    <t>JAGUA</t>
+  </si>
+  <si>
+    <t>KUSKELA</t>
+  </si>
+  <si>
+    <t>MANIGAON</t>
+  </si>
+  <si>
+    <t>MARLAD</t>
+  </si>
+  <si>
+    <t>NAREN</t>
+  </si>
+  <si>
+    <t>PARASARA</t>
+  </si>
+  <si>
+    <t>SIHINI</t>
+  </si>
+  <si>
+    <t>bhalegaon</t>
+  </si>
+  <si>
+    <t>bijepur</t>
+  </si>
+  <si>
+    <t>digsira</t>
+  </si>
+  <si>
     <t>Done</t>
-  </si>
-  <si>
-    <t>DIGSIRA</t>
-  </si>
-  <si>
-    <t>GHANTABAHALI</t>
-  </si>
-  <si>
-    <t>GHODAR</t>
-  </si>
-  <si>
-    <t>JAGUA</t>
-  </si>
-  <si>
-    <t>KUSKELA</t>
-  </si>
-  <si>
-    <t>MANIGAON</t>
-  </si>
-  <si>
-    <t>MARLAD</t>
-  </si>
-  <si>
-    <t>NAREN</t>
-  </si>
-  <si>
-    <t>PARASARA</t>
-  </si>
-  <si>
-    <t>SIHINI</t>
-  </si>
-  <si>
-    <t>bhalegaon</t>
-  </si>
-  <si>
-    <t>bijepur</t>
-  </si>
-  <si>
-    <t>digsira</t>
   </si>
   <si>
     <t>jagua</t>
@@ -744,16 +744,14 @@
       <c r="H2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="1" t="s">
-        <v>15</v>
-      </c>
+      <c r="I2" s="1"/>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
@@ -780,7 +778,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -807,7 +805,7 @@
         <v>9</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>11</v>
@@ -834,7 +832,7 @@
         <v>9</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -861,7 +859,7 @@
         <v>9</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>11</v>
@@ -888,7 +886,7 @@
         <v>9</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>11</v>
@@ -915,7 +913,7 @@
         <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>11</v>
@@ -942,7 +940,7 @@
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>11</v>
@@ -969,7 +967,7 @@
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>11</v>
@@ -996,7 +994,7 @@
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>11</v>
@@ -1023,7 +1021,7 @@
         <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>11</v>
@@ -1050,7 +1048,7 @@
         <v>9</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>11</v>
@@ -1077,28 +1075,28 @@
         <v>9</v>
       </c>
       <c r="B15" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I15" s="2" t="s">
         <v>28</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F15" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G15" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H15" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
@@ -1337,7 +1335,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B6" t="s">
         <v>48</v>
@@ -1348,7 +1346,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" t="s">
         <v>50</v>
@@ -1359,7 +1357,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
         <v>52</v>
@@ -1370,7 +1368,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
         <v>54</v>
@@ -1392,7 +1390,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B11" t="s">
         <v>58</v>
@@ -1403,7 +1401,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
         <v>59</v>
@@ -1414,7 +1412,7 @@
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B13" t="s">
         <v>61</v>
@@ -1425,7 +1423,7 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B14" t="s">
         <v>63</v>
@@ -1436,7 +1434,7 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
         <v>65</v>
@@ -1458,7 +1456,7 @@
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B17" t="s">
         <v>70</v>
@@ -1480,7 +1478,7 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B19" t="s">
         <v>74</v>
@@ -1491,7 +1489,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B20" t="s">
         <v>76</v>
@@ -1502,7 +1500,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B21" t="s">
         <v>78</v>

</xml_diff>

<commit_message>
fixed reconsilation with date
</commit_message>
<xml_diff>
--- a/files/reconsilationfornmat.xlsx
+++ b/files/reconsilationfornmat.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="248" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="87">
   <si>
     <t>BLOCK</t>
   </si>
@@ -38,7 +38,7 @@
     <t>Post office</t>
   </si>
   <si>
-    <t>remarks</t>
+    <t>Last Day Closed</t>
   </si>
   <si>
     <t>TITILAGARH</t>
@@ -59,6 +59,9 @@
     <t>no</t>
   </si>
   <si>
+    <t>04/08/2026</t>
+  </si>
+  <si>
     <t>DIGSIRA</t>
   </si>
   <si>
@@ -95,181 +98,178 @@
     <t>bijepur</t>
   </si>
   <si>
+    <t>kursud</t>
+  </si>
+  <si>
+    <t>luthurbandh</t>
+  </si>
+  <si>
+    <t>mahulpada</t>
+  </si>
+  <si>
+    <t>siluan</t>
+  </si>
+  <si>
+    <t>userid</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>ALANDA</t>
+  </si>
+  <si>
+    <t>PR-ALANDA-V-ADM</t>
+  </si>
+  <si>
+    <t>Alan#1234</t>
+  </si>
+  <si>
+    <t>ADABAHAL</t>
+  </si>
+  <si>
+    <t>PR-ADABAHAL-V-ADM</t>
+  </si>
+  <si>
+    <t>Adab@#234</t>
+  </si>
+  <si>
+    <t>PR-BANDUPALA-V-ADM</t>
+  </si>
+  <si>
+    <t>Band#$234</t>
+  </si>
+  <si>
+    <t>BANJIPADAR</t>
+  </si>
+  <si>
+    <t>PR-BANJIPADAR-V-ADM</t>
+  </si>
+  <si>
+    <t>Admin@2007</t>
+  </si>
+  <si>
+    <t>PR-DIGSIRA-V-ADM</t>
+  </si>
+  <si>
+    <t>Digs@#234</t>
+  </si>
+  <si>
+    <t>PR-GHANTABAHALI-V-ADM</t>
+  </si>
+  <si>
+    <t>Ghant@#234</t>
+  </si>
+  <si>
+    <t>PR-GHODAR-V-ADM</t>
+  </si>
+  <si>
+    <t>Ghod$%234</t>
+  </si>
+  <si>
+    <t>PR-JAGUA-V-ADM</t>
+  </si>
+  <si>
+    <t>Admin@2006</t>
+  </si>
+  <si>
+    <t>KHOLAN</t>
+  </si>
+  <si>
+    <t>PR-KHOLAN-V-ADM</t>
+  </si>
+  <si>
+    <t>PR-KUSKELA-V-ADM</t>
+  </si>
+  <si>
+    <t>PR-MANIGAON-V-ADM</t>
+  </si>
+  <si>
+    <t>Mani#$234</t>
+  </si>
+  <si>
+    <t>PR-MARLAD-V-ADM</t>
+  </si>
+  <si>
+    <t>Marl#$234</t>
+  </si>
+  <si>
+    <t>PR-NAREN-V-ADM</t>
+  </si>
+  <si>
+    <t>Nare@#234</t>
+  </si>
+  <si>
+    <t>PR-PARASARA-V-ADM</t>
+  </si>
+  <si>
+    <t>Para#$234</t>
+  </si>
+  <si>
+    <t>SAGADGHAT</t>
+  </si>
+  <si>
+    <t>PR-SAGADGHAT-V-ADM</t>
+  </si>
+  <si>
+    <t>Saga@#234</t>
+  </si>
+  <si>
+    <t>PR-SIHINI-V1-ADM</t>
+  </si>
+  <si>
+    <t>SILUAN</t>
+  </si>
+  <si>
+    <t>PR-SILUAN-V-ADM</t>
+  </si>
+  <si>
+    <t>Silu#$234</t>
+  </si>
+  <si>
+    <t>pr-bhalegaon-v-adm</t>
+  </si>
+  <si>
+    <t>Bhal@#234</t>
+  </si>
+  <si>
+    <t>pr-bijepur-v-adm</t>
+  </si>
+  <si>
+    <t>Bije#$234</t>
+  </si>
+  <si>
     <t>digsira</t>
   </si>
   <si>
-    <t>Done</t>
+    <t>pr-digsira-v-adm</t>
   </si>
   <si>
     <t>jagua</t>
   </si>
   <si>
-    <t>kursud</t>
-  </si>
-  <si>
-    <t>luthurbandh</t>
-  </si>
-  <si>
-    <t>mahulpada</t>
+    <t>pr-jagua-v-adm</t>
+  </si>
+  <si>
+    <t>Jagu#1234</t>
+  </si>
+  <si>
+    <t>pr-kursud-v-adm</t>
+  </si>
+  <si>
+    <t>Kurs@#123</t>
+  </si>
+  <si>
+    <t>pr-luthurbandh-v-adm</t>
+  </si>
+  <si>
+    <t>Luth$%234</t>
+  </si>
+  <si>
+    <t>pr-mahulpada-v-adm</t>
   </si>
   <si>
     <t>naren</t>
-  </si>
-  <si>
-    <t>siluan</t>
-  </si>
-  <si>
-    <t>userid</t>
-  </si>
-  <si>
-    <t>password</t>
-  </si>
-  <si>
-    <t>ALANDA</t>
-  </si>
-  <si>
-    <t>PR-ALANDA-V-ADM</t>
-  </si>
-  <si>
-    <t>Alan#1234</t>
-  </si>
-  <si>
-    <t>ADABAHAL</t>
-  </si>
-  <si>
-    <t>PR-ADABAHAL-V-ADM</t>
-  </si>
-  <si>
-    <t>Adab@#234</t>
-  </si>
-  <si>
-    <t>PR-BANDUPALA-V-ADM</t>
-  </si>
-  <si>
-    <t>Band#$234</t>
-  </si>
-  <si>
-    <t>BANJIPADAR</t>
-  </si>
-  <si>
-    <t>PR-BANJIPADAR-V-ADM</t>
-  </si>
-  <si>
-    <t>Admin@2007</t>
-  </si>
-  <si>
-    <t>PR-DIGSIRA-V-ADM</t>
-  </si>
-  <si>
-    <t>Digs@#234</t>
-  </si>
-  <si>
-    <t>PR-GHANTABAHALI-V-ADM</t>
-  </si>
-  <si>
-    <t>Ghant@#234</t>
-  </si>
-  <si>
-    <t>PR-GHODAR-V-ADM</t>
-  </si>
-  <si>
-    <t>Ghod$%234</t>
-  </si>
-  <si>
-    <t>PR-JAGUA-V-ADM</t>
-  </si>
-  <si>
-    <t>Admin@2006</t>
-  </si>
-  <si>
-    <t>KHOLAN</t>
-  </si>
-  <si>
-    <t>PR-KHOLAN-V-ADM</t>
-  </si>
-  <si>
-    <t>PR-KUSKELA-V-ADM</t>
-  </si>
-  <si>
-    <t>PR-MANIGAON-V-ADM</t>
-  </si>
-  <si>
-    <t>Mani#$234</t>
-  </si>
-  <si>
-    <t>PR-MARLAD-V-ADM</t>
-  </si>
-  <si>
-    <t>Marl#$234</t>
-  </si>
-  <si>
-    <t>PR-NAREN-V-ADM</t>
-  </si>
-  <si>
-    <t>Nare@#234</t>
-  </si>
-  <si>
-    <t>PR-PARASARA-V-ADM</t>
-  </si>
-  <si>
-    <t>Para#$234</t>
-  </si>
-  <si>
-    <t>SAGADGHAT</t>
-  </si>
-  <si>
-    <t>PR-SAGADGHAT-V-ADM</t>
-  </si>
-  <si>
-    <t>Saga@#234</t>
-  </si>
-  <si>
-    <t>PR-SIHINI-V1-ADM</t>
-  </si>
-  <si>
-    <t>SILUAN</t>
-  </si>
-  <si>
-    <t>PR-SILUAN-V-ADM</t>
-  </si>
-  <si>
-    <t>Silu#$234</t>
-  </si>
-  <si>
-    <t>pr-bhalegaon-v-adm</t>
-  </si>
-  <si>
-    <t>Bhal@#234</t>
-  </si>
-  <si>
-    <t>pr-bijepur-v-adm</t>
-  </si>
-  <si>
-    <t>Bije#$234</t>
-  </si>
-  <si>
-    <t>pr-digsira-v-adm</t>
-  </si>
-  <si>
-    <t>pr-jagua-v-adm</t>
-  </si>
-  <si>
-    <t>Jagu#1234</t>
-  </si>
-  <si>
-    <t>pr-kursud-v-adm</t>
-  </si>
-  <si>
-    <t>Kurs#1234</t>
-  </si>
-  <si>
-    <t>pr-luthurbandh-v-adm</t>
-  </si>
-  <si>
-    <t>Luth$%234</t>
-  </si>
-  <si>
-    <t>pr-mahulpada-v-adm</t>
   </si>
   <si>
     <t>pr-naren-v-adm</t>
@@ -279,7 +279,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -292,6 +292,11 @@
       <name val="Aptos Narrow"/>
     </font>
     <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <name val="Calibri"/>
     </font>
@@ -331,12 +336,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -676,7 +682,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="11.428571428571429" customWidth="1"/>
@@ -687,10 +693,11 @@
     <col min="6" max="6" width="9.285714285714286" customWidth="1"/>
     <col min="7" max="7" width="13.571428571428571" customWidth="1"/>
     <col min="8" max="8" width="9.285714285714286" customWidth="1"/>
-    <col min="9" max="24" width="13.571428571428571" customWidth="1"/>
+    <col min="9" max="9" width="18.857142857142858" customWidth="1"/>
+    <col min="10" max="23" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" ht="15" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -715,11 +722,11 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" ht="19.5" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="2" ht="15.75" customHeight="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>9</v>
       </c>
@@ -744,14 +751,16 @@
       <c r="H2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I2" s="1"/>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>11</v>
@@ -771,14 +780,13 @@
       <c r="H3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I3" s="2"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>11</v>
@@ -798,14 +806,13 @@
       <c r="H4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I4" s="2"/>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>11</v>
@@ -825,14 +832,13 @@
       <c r="H5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I5" s="2"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>11</v>
@@ -852,14 +858,13 @@
       <c r="H6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I6" s="2"/>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>11</v>
@@ -879,14 +884,13 @@
       <c r="H7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I7" s="2"/>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>11</v>
@@ -906,14 +910,13 @@
       <c r="H8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I8" s="2"/>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>11</v>
@@ -933,14 +936,13 @@
       <c r="H9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I9" s="2"/>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C10" s="2" t="s">
         <v>11</v>
@@ -960,14 +962,13 @@
       <c r="H10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I10" s="2"/>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>11</v>
@@ -987,14 +988,13 @@
       <c r="H11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I11" s="2"/>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>11</v>
@@ -1014,14 +1014,13 @@
       <c r="H12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I12" s="2"/>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>11</v>
@@ -1041,14 +1040,13 @@
       <c r="H13" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I13" s="2"/>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>11</v>
@@ -1068,14 +1066,13 @@
       <c r="H14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I14" s="2"/>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>11</v>
@@ -1095,11 +1092,8 @@
       <c r="H15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I15" s="2" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>9</v>
       </c>
@@ -1124,9 +1118,8 @@
       <c r="H16" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I16" s="2"/>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>9</v>
       </c>
@@ -1151,9 +1144,8 @@
       <c r="H17" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I17" s="2"/>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
         <v>9</v>
       </c>
@@ -1178,88 +1170,6 @@
       <c r="H18" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="I18" s="2"/>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B19" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="C19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D19" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E19" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I19" s="2"/>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B20" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E20" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I20" s="2"/>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="B21" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E21" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="H21" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I21" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1278,37 +1188,37 @@
     <col min="4" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>1</v>
       </c>
       <c r="B1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" t="s">
         <v>35</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C2" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="2" ht="18.75" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>37</v>
-      </c>
-      <c r="B2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="C3" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -1316,255 +1226,258 @@
         <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="C7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B8" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C8" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B10" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C11" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B14" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C14" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C15" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B16" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C16" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C17" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C18" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B19" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C19" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C20" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="B21" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="B22" t="s">
+        <v>78</v>
+      </c>
+      <c r="C22" t="s">
         <v>79</v>
-      </c>
-      <c r="C22" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B23" t="s">
+        <v>80</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>81</v>
-      </c>
-      <c r="C23" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B24" t="s">
+        <v>82</v>
+      </c>
+      <c r="C24" t="s">
         <v>83</v>
-      </c>
-      <c r="C24" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B25" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C25" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>33</v>
+        <v>85</v>
       </c>
       <c r="B26" t="s">
         <v>86</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C23" r:id="rId1"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>